<commit_message>
assets: change typo in filename
</commit_message>
<xml_diff>
--- a/assets/Event Import 2026.xlsx
+++ b/assets/Event Import 2026.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11214"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10201"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/gweiher/Sites/die-bruecke-portal/assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93EFA645-04AB-3D4A-A7A5-FD98D2DCB195}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF393540-C4CF-C945-8B35-CAC329D4B186}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2760" yWindow="2900" windowWidth="28240" windowHeight="17240" xr2:uid="{0E41F6F8-BC74-B449-8FE8-D336C1FDB90E}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="58">
   <si>
     <t>title</t>
   </si>
@@ -98,9 +98,6 @@
   </si>
   <si>
     <t>Charly Blaha</t>
-  </si>
-  <si>
-    <t>Lesung mit Musik Internationaler Frauen Tag</t>
   </si>
   <si>
     <t>Sir Oliver &amp; Ripoff</t>
@@ -284,13 +281,27 @@
 Gottfried David Gfrerer: Stimme, Resonatorgitarre, Gitarre
 Foto: Hanna Haidn</t>
   </si>
+  <si>
+    <t>Skin Faxi</t>
+  </si>
+  <si>
+    <t>Skin Faxi sucht mit der Kraft der Tradition von Nyckelharpa (Kurt Bauer), Cello (Vero Gmeindl) und Gesang klare und reduzierte Klangstrukturen und verbindet barocke Klänge mit Minimal Music, Pagan Folk und Contemporary Pop. Ein musikalisches Tableau vivant (an animated map of music).
+Inspiriert von der isländischen Sage des Pferdes mit leuchtender Mähne, das den Tag selbst trägt, lädt die einzigartige Zusammenstellung dazu ein, zeitlose Werke neu zu interpretieren und einzutauchen in vielschichtige Rhythmen und repetitive Muster.
+Reduzierte Klänge und minimalistische Strukturen der kontinuierlich erscheinenden Elemente eröffnet dem Zuhörenden die Möglichkeit loszulassen und zu vergessen, um Skin Faxi am endlosen Horizont tagtäglich von Neuem zu begrüßen.</t>
+  </si>
+  <si>
+    <t>Ich bin Autist:in – Eine Lesung mit musikalischer Begleitung</t>
+  </si>
+  <si>
+    <t>Wir laden euch ganz herzlich ein, einen Abend mit uns zu verbringen, bei dem es vor allem ums Zuhören und Verstehen geht. Unter dem Titel „Ich bin Autist:in“ wollen wir gemeinsam mit euch hinschauen und sensibilisieren. Mag. Daniela Janisch liest aus ihren Texten und wird dabei live von der Grazer Frauenphilharmonie begleitet. Wir finden, diese Mischung aus Lesung und Musik schafft genau den richtigen Rahmen für dieses Thema. Nach dem Programm laufen wir aber nicht gleich auseinander: Bleibt gerne noch da! Wir freuen uns auf Diskussionen, eine Signierstunde oder einfach ein gemütliches Beisammensein mit euch, um den Abend nett ausklingen zu lassen. Wann und wo? Wir treffen uns am Sonntag, den 8. März 2026 um 18:00 Uhr. Ort des Geschehens ist „DIE BRÜCKE“ in der Grabenstraße 39A in Graz. Der Eintritt für den Abend beträgt 25 Euro.</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="168" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
+    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
   </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
@@ -348,7 +359,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -691,11 +702,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{05488E38-2604-B546-A869-B4B325438FF4}">
-  <dimension ref="A1:H38"/>
+  <dimension ref="A1:H39"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="38.1640625" style="2" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="41.1640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="42.5" style="2" customWidth="1"/>
+    <col min="2" max="2" width="29.6640625" style="2" customWidth="1"/>
     <col min="3" max="4" width="18" style="2" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="17" style="2" customWidth="1"/>
     <col min="6" max="6" width="17.5" style="2" customWidth="1"/>
@@ -758,7 +769,7 @@
         <v>12</v>
       </c>
       <c r="B3" s="2" t="str">
-        <f t="shared" ref="B3:B38" si="0">LOWER(SUBSTITUTE(A3," ","-"))</f>
+        <f t="shared" ref="B3:B39" si="0">LOWER(SUBSTITUTE(A3," ","-"))</f>
         <v>oser-steinrück-quartett</v>
       </c>
       <c r="C3" s="3">
@@ -813,37 +824,40 @@
         <v>13</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:8" ht="204" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
-        <v>16</v>
+        <v>54</v>
       </c>
       <c r="B6" s="2" t="str">
         <f t="shared" si="0"/>
-        <v>matthias-kempf</v>
+        <v>skin-faxi</v>
       </c>
       <c r="C6" s="3">
-        <v>46087.833333333336</v>
+        <v>46080.833333333336</v>
       </c>
       <c r="D6" s="3">
-        <v>46087.916666666664</v>
+        <v>46080.916666666664</v>
       </c>
       <c r="F6" s="2" t="s">
         <v>13</v>
+      </c>
+      <c r="G6" s="4" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B7" s="2" t="str">
         <f t="shared" si="0"/>
-        <v>charly-blaha</v>
+        <v>matthias-kempf</v>
       </c>
       <c r="C7" s="3">
-        <v>46088.833333333336</v>
+        <v>46087.833333333336</v>
       </c>
       <c r="D7" s="3">
-        <v>46088.916666666664</v>
+        <v>46087.916666666664</v>
       </c>
       <c r="F7" s="2" t="s">
         <v>13</v>
@@ -851,53 +865,56 @@
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B8" s="2" t="str">
         <f t="shared" si="0"/>
-        <v>lesung-mit-musik-internationaler-frauen-tag</v>
+        <v>charly-blaha</v>
       </c>
       <c r="C8" s="3">
-        <v>46089.708333333336</v>
+        <v>46088.833333333336</v>
       </c>
       <c r="D8" s="3">
-        <v>46089.791666666664</v>
+        <v>46088.916666666664</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>40</v>
+        <v>13</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
-        <v>19</v>
+        <v>56</v>
       </c>
       <c r="B9" s="2" t="str">
         <f t="shared" si="0"/>
-        <v>sir-oliver-&amp;-ripoff</v>
+        <v>ich-bin-autist:in-–-eine-lesung-mit-musikalischer-begleitung</v>
       </c>
       <c r="C9" s="3">
-        <v>46093.833333333336</v>
+        <v>46089.708333333336</v>
       </c>
       <c r="D9" s="3">
-        <v>46093.916666666664</v>
+        <v>46089.791666666664</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>13</v>
+        <v>39</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>57</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B10" s="2" t="str">
         <f t="shared" si="0"/>
-        <v>riccardo-grosso-duo</v>
+        <v>sir-oliver-&amp;-ripoff</v>
       </c>
       <c r="C10" s="3">
-        <v>46095.833333333336</v>
+        <v>46093.833333333336</v>
       </c>
       <c r="D10" s="3">
-        <v>46095.916666666664</v>
+        <v>46093.916666666664</v>
       </c>
       <c r="F10" s="2" t="s">
         <v>13</v>
@@ -905,92 +922,92 @@
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B11" s="2" t="str">
         <f t="shared" si="0"/>
+        <v>riccardo-grosso-duo</v>
+      </c>
+      <c r="C11" s="3">
+        <v>46095.833333333336</v>
+      </c>
+      <c r="D11" s="3">
+        <v>46095.916666666664</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A12" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B12" s="2" t="str">
+        <f t="shared" si="0"/>
         <v>kabarett-cuvee</v>
       </c>
-      <c r="C11" s="3">
+      <c r="C12" s="3">
         <v>46100.833333333336</v>
       </c>
-      <c r="D11" s="3">
+      <c r="D12" s="3">
         <v>46100.916666666664</v>
       </c>
-      <c r="F11" s="2" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" ht="289" x14ac:dyDescent="0.2">
-      <c r="A12" s="1" t="s">
+      <c r="F12" s="2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" ht="289" x14ac:dyDescent="0.2">
+      <c r="A13" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B12" s="2" t="str">
+      <c r="B13" s="2" t="str">
         <f t="shared" si="0"/>
         <v>mord-vor-ort</v>
       </c>
-      <c r="C12" s="3">
+      <c r="C13" s="3">
         <v>46106.791666666664</v>
       </c>
-      <c r="D12" s="3">
+      <c r="D13" s="3">
         <v>46106.875</v>
       </c>
-      <c r="F12" s="2" t="s">
+      <c r="F13" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="G12" s="4" t="s">
+      <c r="G13" s="4" t="s">
         <v>11</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A13" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="B13" s="2" t="str">
-        <f t="shared" si="0"/>
-        <v>homajon-sefat</v>
-      </c>
-      <c r="C13" s="3">
-        <v>46108.833333333336</v>
-      </c>
-      <c r="D13" s="3">
-        <v>46108.916666666664</v>
-      </c>
-      <c r="F13" s="2" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
-        <v>22</v>
+        <v>41</v>
       </c>
       <c r="B14" s="2" t="str">
         <f t="shared" si="0"/>
-        <v>baba-yaga</v>
+        <v>homajon-sefat</v>
       </c>
       <c r="C14" s="3">
-        <v>46122.833333333336</v>
+        <v>46108.833333333336</v>
       </c>
       <c r="D14" s="3">
-        <v>46122.916666666664</v>
+        <v>46108.916666666664</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>13</v>
+        <v>38</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B15" s="2" t="str">
         <f t="shared" si="0"/>
-        <v>manfred-sucher</v>
+        <v>baba-yaga</v>
       </c>
       <c r="C15" s="3">
-        <v>46128.833333333336</v>
+        <v>46122.833333333336</v>
       </c>
       <c r="D15" s="3">
-        <v>46128.916666666664</v>
+        <v>46122.916666666664</v>
       </c>
       <c r="F15" s="2" t="s">
         <v>13</v>
@@ -998,455 +1015,476 @@
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A16" s="1" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B16" s="2" t="str">
         <f t="shared" si="0"/>
+        <v>manfred-sucher</v>
+      </c>
+      <c r="C16" s="3">
+        <v>46128.833333333336</v>
+      </c>
+      <c r="D16" s="3">
+        <v>46128.916666666664</v>
+      </c>
+      <c r="F16" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A17" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B17" s="2" t="str">
+        <f t="shared" si="0"/>
         <v>nette-eltere-herren</v>
       </c>
-      <c r="C16" s="3">
+      <c r="C17" s="3">
         <v>46129.833333333336</v>
       </c>
-      <c r="D16" s="3">
+      <c r="D17" s="3">
         <v>46129.916666666664</v>
       </c>
-      <c r="F16" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" ht="289" x14ac:dyDescent="0.2">
-      <c r="A17" s="1" t="s">
+      <c r="F17" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" ht="289" x14ac:dyDescent="0.2">
+      <c r="A18" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B17" s="2" t="str">
+      <c r="B18" s="2" t="str">
         <f t="shared" si="0"/>
         <v>mord-vor-ort</v>
       </c>
-      <c r="C17" s="3">
+      <c r="C18" s="3">
         <v>46134.791666666664</v>
       </c>
-      <c r="D17" s="3">
+      <c r="D18" s="3">
         <v>46134.875</v>
       </c>
-      <c r="F17" s="2" t="s">
+      <c r="F18" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="G17" s="4" t="s">
+      <c r="G18" s="4" t="s">
         <v>11</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A18" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="B18" s="2" t="str">
-        <f t="shared" si="0"/>
-        <v>mally-&amp;-biber-hermann</v>
-      </c>
-      <c r="C18" s="3">
-        <v>46135.833333333336</v>
-      </c>
-      <c r="D18" s="3">
-        <v>46135.916666666664</v>
-      </c>
-      <c r="F18" s="2" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A19" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B19" s="2" t="str">
+        <f t="shared" si="0"/>
+        <v>mally-&amp;-biber-hermann</v>
+      </c>
+      <c r="C19" s="3">
+        <v>46135.833333333336</v>
+      </c>
+      <c r="D19" s="3">
+        <v>46135.916666666664</v>
+      </c>
+      <c r="F19" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A20" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B20" s="2" t="str">
+        <f t="shared" si="0"/>
+        <v>son-of-the-velvet-rat</v>
+      </c>
+      <c r="C20" s="3">
+        <v>46136.833333333336</v>
+      </c>
+      <c r="D20" s="3">
+        <v>46136.916666666664</v>
+      </c>
+      <c r="F20" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" ht="388" x14ac:dyDescent="0.2">
+      <c r="A21" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B19" s="2" t="str">
-        <f t="shared" si="0"/>
-        <v>son-of-the-velvet-rat</v>
-      </c>
-      <c r="C19" s="3">
-        <v>46136.833333333336</v>
-      </c>
-      <c r="D19" s="3">
-        <v>46136.916666666664</v>
-      </c>
-      <c r="F19" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" ht="388" x14ac:dyDescent="0.2">
-      <c r="A20" s="1" t="s">
+      <c r="B21" s="2" t="str">
+        <f t="shared" si="0"/>
+        <v>solarkreis</v>
+      </c>
+      <c r="C21" s="3">
+        <v>46137.833333333336</v>
+      </c>
+      <c r="D21" s="3">
+        <v>46137.916666666664</v>
+      </c>
+      <c r="F21" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G21" s="4" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" ht="216" x14ac:dyDescent="0.2">
+      <c r="A22" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="B20" s="2" t="str">
-        <f t="shared" si="0"/>
-        <v>solarkreis</v>
-      </c>
-      <c r="C20" s="3">
-        <v>46137.833333333336</v>
-      </c>
-      <c r="D20" s="3">
-        <v>46137.916666666664</v>
-      </c>
-      <c r="F20" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G20" s="4" t="s">
+      <c r="B22" s="2" t="str">
+        <f t="shared" si="0"/>
+        <v>chordovoice</v>
+      </c>
+      <c r="C22" s="3">
+        <v>46142.833333333336</v>
+      </c>
+      <c r="D22" s="3">
+        <v>46142.916666666664</v>
+      </c>
+      <c r="F22" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G22" s="5" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="21" spans="1:7" ht="216" x14ac:dyDescent="0.2">
-      <c r="A21" s="1" t="s">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A23" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B21" s="2" t="str">
-        <f t="shared" si="0"/>
-        <v>chordovoice</v>
-      </c>
-      <c r="C21" s="3">
-        <v>46142.833333333336</v>
-      </c>
-      <c r="D21" s="3">
-        <v>46142.916666666664</v>
-      </c>
-      <c r="F21" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G21" s="5" t="s">
+      <c r="B23" s="2" t="str">
+        <f t="shared" si="0"/>
+        <v>philipp-grießler/andreas-johann-bauer</v>
+      </c>
+      <c r="C23" s="3">
+        <v>46150.833333333336</v>
+      </c>
+      <c r="D23" s="3">
+        <v>46150.916666666664</v>
+      </c>
+      <c r="F23" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" ht="289" x14ac:dyDescent="0.2">
+      <c r="A24" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B24" s="2" t="str">
+        <f t="shared" si="0"/>
+        <v>mord-vor-ort</v>
+      </c>
+      <c r="C24" s="3">
+        <v>46169.791666666664</v>
+      </c>
+      <c r="D24" s="3">
+        <v>46169.875</v>
+      </c>
+      <c r="F24" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G24" s="4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" ht="409" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A25" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B25" s="2" t="str">
+        <f t="shared" si="0"/>
+        <v>hans-theessink</v>
+      </c>
+      <c r="C25" s="3">
+        <v>46184.8125</v>
+      </c>
+      <c r="D25" s="3">
+        <v>46184.916666666664</v>
+      </c>
+      <c r="F25" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G25" s="4" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A22" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="B22" s="2" t="str">
-        <f t="shared" si="0"/>
-        <v>philipp-grießler/andreas-johann-bauer</v>
-      </c>
-      <c r="C22" s="3">
-        <v>46150.833333333336</v>
-      </c>
-      <c r="D22" s="3">
-        <v>46150.916666666664</v>
-      </c>
-      <c r="F22" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" ht="289" x14ac:dyDescent="0.2">
-      <c r="A23" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B23" s="2" t="str">
-        <f t="shared" si="0"/>
-        <v>mord-vor-ort</v>
-      </c>
-      <c r="C23" s="3">
-        <v>46169.791666666664</v>
-      </c>
-      <c r="D23" s="3">
-        <v>46169.875</v>
-      </c>
-      <c r="F23" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="G23" s="4" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7" ht="409" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="1" t="s">
+    <row r="26" spans="1:7" ht="119" x14ac:dyDescent="0.2">
+      <c r="A26" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B26" s="2" t="str">
+        <f t="shared" si="0"/>
+        <v>rosetti-sisters</v>
+      </c>
+      <c r="C26" s="3">
+        <v>46192.8125</v>
+      </c>
+      <c r="D26" s="3">
+        <v>46192.916666666664</v>
+      </c>
+      <c r="F26" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G26" s="4" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A27" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="B24" s="2" t="str">
-        <f t="shared" si="0"/>
-        <v>hans-theessink</v>
-      </c>
-      <c r="C24" s="3">
-        <v>46184.8125</v>
-      </c>
-      <c r="D24" s="3">
-        <v>46184.916666666664</v>
-      </c>
-      <c r="F24" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G24" s="4" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7" ht="119" x14ac:dyDescent="0.2">
-      <c r="A25" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="B25" s="2" t="str">
-        <f t="shared" si="0"/>
-        <v>rosetti-sisters</v>
-      </c>
-      <c r="C25" s="3">
-        <v>46192.8125</v>
-      </c>
-      <c r="D25" s="3">
-        <v>46192.916666666664</v>
-      </c>
-      <c r="F25" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G25" s="4" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A26" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="B26" s="2" t="str">
+      <c r="B27" s="2" t="str">
         <f t="shared" si="0"/>
         <v>abba-4-you</v>
       </c>
-      <c r="C26" s="3">
+      <c r="C27" s="3">
         <v>46193.833333333336</v>
       </c>
-      <c r="D26" s="3">
+      <c r="D27" s="3">
         <v>46193.916666666664</v>
       </c>
-      <c r="F26" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="27" spans="1:7" ht="289" x14ac:dyDescent="0.2">
-      <c r="A27" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B27" s="2" t="str">
-        <f t="shared" si="0"/>
-        <v>mord-vor-ort</v>
-      </c>
-      <c r="C27" s="3">
-        <v>46197.791666666664</v>
-      </c>
-      <c r="D27" s="3">
-        <v>46197.875</v>
-      </c>
       <c r="F27" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="G27" s="4" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="28" spans="1:7" ht="289" x14ac:dyDescent="0.2">
       <c r="A28" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B28" s="2" t="str">
+        <f t="shared" si="0"/>
+        <v>mord-vor-ort</v>
+      </c>
+      <c r="C28" s="3">
+        <v>46197.791666666664</v>
+      </c>
+      <c r="D28" s="3">
+        <v>46197.875</v>
+      </c>
+      <c r="F28" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G28" s="4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" ht="289" x14ac:dyDescent="0.2">
+      <c r="A29" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="B29" s="2" t="str">
+        <f t="shared" si="0"/>
+        <v>boxty</v>
+      </c>
+      <c r="C29" s="3">
+        <v>46199.8125</v>
+      </c>
+      <c r="D29" s="3">
+        <v>46199.916666666664</v>
+      </c>
+      <c r="F29" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G29" s="4" t="s">
         <v>47</v>
-      </c>
-      <c r="B28" s="2" t="str">
-        <f t="shared" si="0"/>
-        <v>boxty</v>
-      </c>
-      <c r="C28" s="3">
-        <v>46199.8125</v>
-      </c>
-      <c r="D28" s="3">
-        <v>46199.916666666664</v>
-      </c>
-      <c r="F28" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G28" s="4" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A29" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="B29" s="2" t="str">
-        <f t="shared" si="0"/>
-        <v>sir-oliver-mally,-peter-schneider,-martin-burböck</v>
-      </c>
-      <c r="C29" s="3">
-        <v>46207.8125</v>
-      </c>
-      <c r="D29" s="3">
-        <v>46207.916666666664</v>
-      </c>
-      <c r="F29" s="2" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A30" s="1" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="B30" s="2" t="str">
         <f t="shared" si="0"/>
-        <v>kabarett-cuvée-sommer-festival-tag-1</v>
+        <v>sir-oliver-mally,-peter-schneider,-martin-burböck</v>
       </c>
       <c r="C30" s="3">
-        <v>46219.8125</v>
+        <v>46207.8125</v>
       </c>
       <c r="D30" s="3">
-        <v>46219.916666666664</v>
+        <v>46207.916666666664</v>
       </c>
       <c r="F30" s="2" t="s">
-        <v>39</v>
+        <v>13</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A31" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B31" s="2" t="str">
         <f t="shared" si="0"/>
-        <v>kabarett-cuvée-sommer-festival-tag-2</v>
+        <v>kabarett-cuvée-sommer-festival-tag-1</v>
       </c>
       <c r="C31" s="3">
-        <v>46220.8125</v>
+        <v>46219.8125</v>
       </c>
       <c r="D31" s="3">
-        <v>46220.916666666664</v>
+        <v>46219.916666666664</v>
       </c>
       <c r="F31" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A32" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B32" s="2" t="str">
+        <f t="shared" si="0"/>
+        <v>kabarett-cuvée-sommer-festival-tag-2</v>
+      </c>
+      <c r="C32" s="3">
+        <v>46220.8125</v>
+      </c>
+      <c r="D32" s="3">
+        <v>46220.916666666664</v>
+      </c>
+      <c r="F32" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="B32" s="2" t="str">
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A33" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B33" s="2" t="str">
         <f t="shared" si="0"/>
         <v>kabarett-cuvée-sommer-festival-tag-3</v>
       </c>
-      <c r="C32" s="3">
+      <c r="C33" s="3">
         <v>46221.8125</v>
       </c>
-      <c r="D32" s="3">
+      <c r="D33" s="3">
         <v>46221.916666666664</v>
       </c>
-      <c r="F32" s="2" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="33" spans="1:7" ht="306" x14ac:dyDescent="0.2">
-      <c r="A33" s="2" t="s">
+      <c r="F33" s="2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" ht="306" x14ac:dyDescent="0.2">
+      <c r="A34" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="B34" s="2" t="str">
+        <f t="shared" si="0"/>
+        <v>ulli-bäer,-matthias-kempf-und-andy-baum-–-ein-abend-zu-dritt</v>
+      </c>
+      <c r="C34" s="3">
+        <v>46227.8125</v>
+      </c>
+      <c r="D34" s="3">
+        <v>46227.916666666664</v>
+      </c>
+      <c r="F34" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G34" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="B33" s="2" t="str">
-        <f t="shared" si="0"/>
-        <v>ulli-bäer,-matthias-kempf-und-andy-baum-–-ein-abend-zu-dritt</v>
-      </c>
-      <c r="C33" s="3">
-        <v>46227.8125</v>
-      </c>
-      <c r="D33" s="3">
-        <v>46227.916666666664</v>
-      </c>
-      <c r="F33" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G33" s="4" t="s">
+    </row>
+    <row r="35" spans="1:7" ht="404" x14ac:dyDescent="0.2">
+      <c r="A35" s="1" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="34" spans="1:7" ht="409.6" x14ac:dyDescent="0.2">
-      <c r="A34" s="1" t="s">
+      <c r="B35" s="2" t="str">
+        <f t="shared" si="0"/>
+        <v>charlie-&amp;-die-kaischlabuam</v>
+      </c>
+      <c r="C35" s="3">
+        <v>46234.8125</v>
+      </c>
+      <c r="D35" s="3">
+        <v>46234.916666666664</v>
+      </c>
+      <c r="F35" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G35" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="B34" s="2" t="str">
-        <f t="shared" si="0"/>
-        <v>charlie-&amp;-die-kaischlabuam</v>
-      </c>
-      <c r="C34" s="3">
-        <v>46234.8125</v>
-      </c>
-      <c r="D34" s="3">
-        <v>46234.916666666664</v>
-      </c>
-      <c r="F34" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G34" s="4" t="s">
+    </row>
+    <row r="36" spans="1:7" ht="170" x14ac:dyDescent="0.2">
+      <c r="A36" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B36" s="2" t="str">
+        <f t="shared" si="0"/>
+        <v>crossing-strings</v>
+      </c>
+      <c r="C36" s="3">
+        <v>46339.833333333336</v>
+      </c>
+      <c r="D36" s="3">
+        <v>46339.916666666664</v>
+      </c>
+      <c r="F36" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G36" s="4" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="35" spans="1:7" ht="187" x14ac:dyDescent="0.2">
-      <c r="A35" s="1" t="s">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A37" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B37" s="2" t="str">
+        <f t="shared" si="0"/>
+        <v>kabarett-cuvee</v>
+      </c>
+      <c r="C37" s="3">
+        <v>46345.833333333336</v>
+      </c>
+      <c r="D37" s="3">
+        <v>46345.916666666664</v>
+      </c>
+      <c r="F37" s="2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" ht="306" x14ac:dyDescent="0.2">
+      <c r="A38" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="B35" s="2" t="str">
-        <f t="shared" si="0"/>
-        <v>crossing-strings</v>
-      </c>
-      <c r="C35" s="3">
-        <v>46339.833333333336</v>
-      </c>
-      <c r="D35" s="3">
-        <v>46339.916666666664</v>
-      </c>
-      <c r="F35" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G35" s="4" t="s">
+      <c r="B38" s="2" t="str">
+        <f t="shared" si="0"/>
+        <v>gottfried-d.-gfrerer</v>
+      </c>
+      <c r="C38" s="3">
+        <v>46346.833333333336</v>
+      </c>
+      <c r="D38" s="3">
+        <v>46346.916666666664</v>
+      </c>
+      <c r="F38" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G38" s="4" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A36" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="B36" s="2" t="str">
-        <f t="shared" si="0"/>
-        <v>kabarett-cuvee</v>
-      </c>
-      <c r="C36" s="3">
-        <v>46345.833333333336</v>
-      </c>
-      <c r="D36" s="3">
-        <v>46345.916666666664</v>
-      </c>
-      <c r="F36" s="2" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="37" spans="1:7" ht="306" x14ac:dyDescent="0.2">
-      <c r="A37" s="1" t="s">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A39" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="B37" s="2" t="str">
-        <f t="shared" si="0"/>
-        <v>gottfried-d.-gfrerer</v>
-      </c>
-      <c r="C37" s="3">
-        <v>46346.833333333336</v>
-      </c>
-      <c r="D37" s="3">
-        <v>46346.916666666664</v>
-      </c>
-      <c r="F37" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G37" s="4" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A38" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="B38" s="2" t="str">
+      <c r="B39" s="2" t="str">
         <f t="shared" si="0"/>
         <v>erwin-r</v>
       </c>
-      <c r="C38" s="3">
+      <c r="C39" s="3">
         <v>46353.8125</v>
       </c>
-      <c r="D38" s="3">
+      <c r="D39" s="3">
         <v>46353.916666666664</v>
       </c>
-      <c r="F38" s="2" t="s">
+      <c r="F39" s="2" t="s">
         <v>13</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A9" r:id="rId1" display="https://diebruecke.social/cms/event-kalender/" xr:uid="{8841008E-1B65-614B-AD0A-708922009ECE}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>